<commit_message>
feat: dynamic JOURS_COLS detection + updated template vierge
- Add _detect_jours_cols() to auto-detect date columns from embedded template
- JOURS_COLS now computed at startup ([2,16,34,46]) instead of hardcoded ([2,18,38,54])
- Re-encode template_vierge_SEPTEMBRE_2026_corrige.xlsx with removed classes
- Remove obsolete files (Jean templates, REF template, old template vierge)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Template_tableau_formateurs_Pierre.xlsx
+++ b/Template_tableau_formateurs_Pierre.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Matheo.DISTINGUIN\Desktop\Rentre_2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4C0735C7-840D-4437-B842-942F37AB4E31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB8377CD-9446-4710-BFD1-2C12874F4342}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-5730" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AFFECTATIONS" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,6 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">AFFECTATIONS!$A$3:$G$13</definedName>
   </definedNames>
   <calcPr calcId="0"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
@@ -140,7 +139,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="40">
   <si>
     <t>AFFECTATIONS FORMATEURS — Rentrée 2025-2026</t>
   </si>
@@ -254,6 +253,12 @@
   </si>
   <si>
     <t>Info</t>
+  </si>
+  <si>
+    <t>BAC PRO 28</t>
+  </si>
+  <si>
+    <t>Maths</t>
   </si>
 </sst>
 </file>
@@ -273,27 +278,32 @@
       <sz val="14"/>
       <color rgb="FF1F4E79"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="9"/>
       <color rgb="FF595959"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="9">
@@ -821,13 +831,25 @@
       </c>
     </row>
     <row r="5" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="6"/>
-      <c r="B5" s="6"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="8"/>
+      <c r="A5" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="D5" s="7">
+        <v>35</v>
+      </c>
+      <c r="E5" s="8">
+        <v>1</v>
+      </c>
       <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
+      <c r="G5" s="6" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="6" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="6"/>

</xml_diff>